<commit_message>
feat(excel): add dynamic identification type, gender, and professional details mapping
</commit_message>
<xml_diff>
--- a/Muestra_Datos_Rocita_50.xlsx
+++ b/Muestra_Datos_Rocita_50.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,7 +426,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Cedula</t>
+          <t>Documento</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -437,6 +437,16 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>Correo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Tipo Documento</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Sexo</t>
         </is>
       </c>
     </row>
@@ -461,6 +471,16 @@
           <t>camila.rivera@correo.com</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -483,6 +503,16 @@
           <t>natalia.cruz@correo.com</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -505,6 +535,16 @@
           <t>patricia.ramirez@correo.com</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -527,6 +567,16 @@
           <t>oscar.sanchez@correo.com</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -549,6 +599,16 @@
           <t>fernanda.gomez@correo.com</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -571,6 +631,16 @@
           <t>carlos.lopez@correo.com</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -593,6 +663,16 @@
           <t>laura.torres@correo.com</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -615,6 +695,16 @@
           <t>mauricio.ortiz@correo.com</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -637,6 +727,16 @@
           <t>ignacio.gutierrez@correo.com</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -659,6 +759,16 @@
           <t>ignacio.flores@correo.com</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -681,6 +791,16 @@
           <t>karla.bravo@correo.com</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -703,6 +823,16 @@
           <t>ricardo.garcia@correo.com</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -725,6 +855,16 @@
           <t>oscar.rivera@correo.com</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -747,6 +887,16 @@
           <t>valentina.torres@correo.com</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -769,6 +919,16 @@
           <t>laura.perez@correo.com</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -791,6 +951,16 @@
           <t>julia.sanchez@correo.com</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -813,6 +983,16 @@
           <t>kevin.lopez@correo.com</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -835,6 +1015,16 @@
           <t>ignacio.castillo@correo.com</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -857,6 +1047,16 @@
           <t>beatriz.rivera@correo.com</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -879,6 +1079,16 @@
           <t>andres.cruz@correo.com</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -901,6 +1111,16 @@
           <t>felipe.diaz@correo.com</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -923,6 +1143,16 @@
           <t>felipe.martinez@correo.com</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -945,6 +1175,16 @@
           <t>beatriz.perez@correo.com</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -967,6 +1207,16 @@
           <t>daniel.rodriguez@correo.com</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -989,6 +1239,16 @@
           <t>kevin.torres@correo.com</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1011,6 +1271,16 @@
           <t>diana.bravo@correo.com</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1033,6 +1303,16 @@
           <t>mauricio.diaz@correo.com</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1055,6 +1335,16 @@
           <t>ignacio.ortiz@correo.com</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1077,6 +1367,16 @@
           <t>natalia.gutierrez@correo.com</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1099,6 +1399,16 @@
           <t>helena.ramirez@correo.com</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1121,6 +1431,16 @@
           <t>camila.martinez@correo.com</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1143,6 +1463,16 @@
           <t>valentina.lopez@correo.com</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1165,6 +1495,16 @@
           <t>natalia.flores@correo.com</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1187,6 +1527,16 @@
           <t>daniel.rojas@correo.com</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1209,6 +1559,16 @@
           <t>natalia.gutierrez@correo.com</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1231,6 +1591,16 @@
           <t>jorge.lopez@correo.com</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1253,6 +1623,16 @@
           <t>camila.torres@correo.com</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1275,6 +1655,16 @@
           <t>fernanda.sanchez@correo.com</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1297,6 +1687,16 @@
           <t>andres.perez@correo.com</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1319,6 +1719,16 @@
           <t>daniel.torres@correo.com</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1341,6 +1751,16 @@
           <t>tomas.garcia@correo.com</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1363,6 +1783,16 @@
           <t>patricia.rodriguez@correo.com</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1385,6 +1815,16 @@
           <t>eduardo.rivera@correo.com</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1407,6 +1847,16 @@
           <t>eduardo.morales@correo.com</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1429,6 +1879,16 @@
           <t>sofia.ortiz@correo.com</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1451,6 +1911,16 @@
           <t>diana.ortiz@correo.com</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1473,6 +1943,16 @@
           <t>patricia.rodriguez@correo.com</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1495,6 +1975,16 @@
           <t>elena.ortiz@correo.com</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1517,6 +2007,16 @@
           <t>camila.ortiz@correo.com</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1537,6 +2037,16 @@
       <c r="D51" t="inlineStr">
         <is>
           <t>diana.cruz@correo.com</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -1551,7 +2061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1570,6 +2080,16 @@
           <t>Lugar de Atencion</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Celular</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1587,6 +2107,16 @@
           <t>Sede Sur - Portal Norte</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>beatriz.perez@consultorio.com</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>+57 311 987 6002</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1604,6 +2134,16 @@
           <t>Sede Centro - Cra 10</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>patricia.perez@consultorio.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>+57 311 987 6003</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1621,6 +2161,16 @@
           <t>Sede Norte - Calle 127</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>carlos.flores@consultorio.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>+57 311 987 6004</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1638,6 +2188,16 @@
           <t>Sede Norte - Calle 127</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>gabriel.ramirez@consultorio.com</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>+57 311 987 6005</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1655,6 +2215,16 @@
           <t>Sede Centro - Cra 10</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>patricia.rojas@consultorio.com</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>+57 311 987 6006</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1672,6 +2242,16 @@
           <t>Sede Sur - Portal Norte</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>alejandro.morales@consultorio.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>+57 311 987 6007</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1689,6 +2269,16 @@
           <t>Sede Sur - Portal Norte</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>diana.rodriguez@consultorio.com</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>+57 311 987 6008</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1706,6 +2296,16 @@
           <t>Sede Norte - Calle 127</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>gabriel.rojas@consultorio.com</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>+57 311 987 6009</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1723,6 +2323,16 @@
           <t>Sede Sur - Portal Norte</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>hugo.flores@consultorio.com</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>+57 311 987 6010</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1738,6 +2348,16 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>Sede Centro - Cra 10</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ignacio.sanchez@consultorio.com</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>+57 311 987 6011</t>
         </is>
       </c>
     </row>
@@ -1752,7 +2372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1763,7 +2383,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Paciente</t>
+          <t>Documento Paciente</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1779,6 +2399,16 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>Lugar</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Nombre Paciente</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Sexo Paciente</t>
         </is>
       </c>
     </row>
@@ -1790,22 +2420,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>1062856493</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Dr. Beatriz Perez</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-05-25 10:00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Sede Sur - Portal Norte</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Camila Rivera</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Dr. Beatriz Perez</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-05-25 10:00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Sede Sur - Portal Norte</t>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -1817,22 +2457,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>1013663970</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Dr. Diana Rodriguez</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:00</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Clínica 100Digital</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Natalia Cruz</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Dr. Diana Rodriguez</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-05-27 12:00</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Clínica 100Digital</t>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -1844,22 +2494,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>1044593454</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Dr. Alejandro Morales</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Clínica 100Digital</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>Patricia Ramirez</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Dr. Alejandro Morales</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-05-21 18:00</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Clínica 100Digital</t>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -1871,22 +2531,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>1021310412</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Dr. Alejandro Morales</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-05-22 08:00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Clínica 100Digital</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>Oscar Sanchez</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Dr. Alejandro Morales</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-05-22 08:00</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Clínica 100Digital</t>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -1898,22 +2568,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>1029636478</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Dr. Alejandro Morales</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-05-26 08:30</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Sede Sur - Portal Norte</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>Fernanda Gomez</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Dr. Alejandro Morales</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2026-05-26 08:30</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Sede Sur - Portal Norte</t>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -1925,22 +2605,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>1071076251</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Dr. Diana Rodriguez</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-05-21 12:00</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Sede Centro - Cra 10</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>Carlos Lopez</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Dr. Diana Rodriguez</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2026-05-21 12:00</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Sede Centro - Cra 10</t>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -1952,22 +2642,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>1037491059</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Dr. Beatriz Perez</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-05-22 15:00</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Clínica 100Digital</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>Laura Torres</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Dr. Beatriz Perez</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-05-22 15:00</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Clínica 100Digital</t>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -1979,22 +2679,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>1076890007</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Dr. Diana Rodriguez</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-05-23 17:30</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>Mauricio Ortiz</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Dr. Diana Rodriguez</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2026-05-23 17:30</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2006,22 +2716,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>1086469987</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Dr. Carlos Flores</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-05-21 17:00</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Sede Centro - Cra 10</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>Ignacio Gutierrez</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Dr. Carlos Flores</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2026-05-21 17:00</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Sede Centro - Cra 10</t>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2033,22 +2753,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>1066699847</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Dr. Ignacio Sanchez</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-05-21 08:00</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sede Sur - Portal Norte</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>Ignacio Flores</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Dr. Ignacio Sanchez</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2026-05-21 08:00</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Sede Sur - Portal Norte</t>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2060,22 +2790,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>1043250775</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Dr. Hugo Flores</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-05-20 10:00</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Clínica 100Digital</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>Karla Bravo</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Dr. Hugo Flores</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2026-05-20 10:00</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Clínica 100Digital</t>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2087,22 +2827,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>1031095711</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Dr. Beatriz Perez</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-05-23 07:30</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sede Centro - Cra 10</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>Ricardo Garcia</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Dr. Beatriz Perez</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2026-05-23 07:30</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Sede Centro - Cra 10</t>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2114,22 +2864,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>1031796573</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Dr. Alejandro Morales</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:30</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Sede Centro - Cra 10</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>Oscar Rivera</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Dr. Alejandro Morales</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2026-05-20 18:30</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Sede Centro - Cra 10</t>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2141,22 +2901,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>1039990355</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Dr. Patricia Rojas</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-05-27 16:00</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>Valentina Torres</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Dr. Patricia Rojas</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2026-05-27 16:00</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2168,22 +2938,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>1060709043</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Dr. Hugo Flores</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:00</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>Laura Perez</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Dr. Hugo Flores</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>2026-05-22 13:00</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -2195,22 +2975,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>1072405842</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Dr. Patricia Rojas</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-05-22 10:30</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Sede Sur - Portal Norte</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>Julia Sanchez</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Dr. Patricia Rojas</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>2026-05-22 10:30</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Sede Sur - Portal Norte</t>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2222,22 +3012,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>1065864295</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Dr. Diana Rodriguez</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2026-05-26 14:30</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Sede Centro - Cra 10</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>Kevin Lopez</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Dr. Diana Rodriguez</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>2026-05-26 14:30</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Sede Centro - Cra 10</t>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2249,22 +3049,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>1080457966</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Dr. Ignacio Sanchez</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-05-20 16:00</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Clínica 100Digital</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>Ignacio Castillo</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Dr. Ignacio Sanchez</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>2026-05-20 16:00</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Clínica 100Digital</t>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2276,22 +3086,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>1058932145</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Dr. Alejandro Morales</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026-05-24 13:00</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Sede Centro - Cra 10</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>Beatriz Rivera</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Dr. Alejandro Morales</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>2026-05-24 13:00</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Sede Centro - Cra 10</t>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -2303,22 +3123,32 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>1093795979</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Dr. Carlos Flores</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2026-05-20 17:00</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>Andres Cruz</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Dr. Carlos Flores</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>2026-05-20 17:00</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2330,22 +3160,32 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>1087691556</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Dr. Hugo Flores</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2026-05-20 16:30</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>Felipe Diaz</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Dr. Hugo Flores</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>2026-05-20 16:30</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2357,22 +3197,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>1076642439</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Dr. Beatriz Perez</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2026-05-20 15:30</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Sede Centro - Cra 10</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>Felipe Martinez</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Dr. Beatriz Perez</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>2026-05-20 15:30</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Sede Centro - Cra 10</t>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2384,22 +3234,32 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>1016345772</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Dr. Hugo Flores</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2026-05-20 18:00</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
           <t>Beatriz Perez</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Dr. Hugo Flores</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>2026-05-20 18:00</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -2411,22 +3271,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>1059217766</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Dr. Hugo Flores</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2026-05-21 09:30</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Sede Centro - Cra 10</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
           <t>Daniel Rodriguez</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Dr. Hugo Flores</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>2026-05-21 09:30</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Sede Centro - Cra 10</t>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2438,22 +3308,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>1033177575</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Dr. Patricia Perez</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2026-05-26 12:00</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Clínica 100Digital</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
           <t>Kevin Torres</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Dr. Patricia Perez</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>2026-05-26 12:00</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Clínica 100Digital</t>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2465,22 +3345,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>1061853019</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Dr. Alejandro Morales</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2026-05-22 17:30</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Clínica 100Digital</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
           <t>Diana Bravo</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Dr. Alejandro Morales</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>2026-05-22 17:30</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Clínica 100Digital</t>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -2492,22 +3382,32 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>1052124918</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Dr. Gabriel Ramirez</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2026-05-20 08:30</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Clínica 100Digital</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
           <t>Mauricio Diaz</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Dr. Gabriel Ramirez</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>2026-05-20 08:30</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Clínica 100Digital</t>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2519,22 +3419,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>1090698154</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Dr. Gabriel Rojas</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2026-05-22 18:00</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Sede Centro - Cra 10</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
           <t>Ignacio Ortiz</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Dr. Gabriel Rojas</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>2026-05-22 18:00</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Sede Centro - Cra 10</t>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2546,22 +3456,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>1040693165</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Dr. Hugo Flores</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2026-05-20 16:00</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Sede Sur - Portal Norte</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
           <t>Natalia Gutierrez</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Dr. Hugo Flores</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>2026-05-20 16:00</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Sede Sur - Portal Norte</t>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -2573,22 +3493,32 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>1085978802</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Dr. Gabriel Rojas</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2026-05-24 14:00</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
           <t>Helena Ramirez</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Dr. Gabriel Rojas</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>2026-05-24 14:00</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -2600,22 +3530,32 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t>1047524946</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Dr. Carlos Flores</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2026-05-25 11:30</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
           <t>Camila Martinez</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Dr. Carlos Flores</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>2026-05-25 11:30</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -2627,22 +3567,32 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>1091206689</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Dr. Gabriel Rojas</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2026-05-24 14:00</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sede Centro - Cra 10</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
           <t>Valentina Lopez</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Dr. Gabriel Rojas</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>2026-05-24 14:00</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Sede Centro - Cra 10</t>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2654,22 +3604,32 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>1054075437</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Dr. Gabriel Rojas</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2026-05-21 12:00</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Sede Centro - Cra 10</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
           <t>Natalia Flores</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Dr. Gabriel Rojas</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>2026-05-21 12:00</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Sede Centro - Cra 10</t>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -2681,22 +3641,32 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>1059071867</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Dr. Patricia Rojas</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2026-05-23 11:30</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
           <t>Daniel Rojas</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Dr. Patricia Rojas</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>2026-05-23 11:30</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2708,22 +3678,32 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>1040693165</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Dr. Beatriz Perez</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2026-05-25 08:30</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Sede Sur - Portal Norte</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
           <t>Natalia Gutierrez</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Dr. Beatriz Perez</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>2026-05-25 08:30</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Sede Sur - Portal Norte</t>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -2735,22 +3715,32 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>1054443779</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Dr. Ignacio Sanchez</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2026-05-24 10:30</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
           <t>Jorge Lopez</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Dr. Ignacio Sanchez</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>2026-05-24 10:30</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2762,22 +3752,32 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>1025014162</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Dr. Patricia Rojas</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2026-05-25 07:00</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Sede Centro - Cra 10</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
           <t>Camila Torres</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Dr. Patricia Rojas</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>2026-05-25 07:00</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Sede Centro - Cra 10</t>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -2789,22 +3789,32 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>1029679342</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Dr. Alejandro Morales</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2026-05-21 16:00</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Clínica 100Digital</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
           <t>Fernanda Sanchez</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Dr. Alejandro Morales</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>2026-05-21 16:00</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Clínica 100Digital</t>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2816,22 +3826,32 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>1021830137</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Dr. Diana Rodriguez</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2026-05-27 17:00</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
           <t>Andres Perez</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Dr. Diana Rodriguez</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>2026-05-27 17:00</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2843,22 +3863,32 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>1019563085</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Dr. Diana Rodriguez</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2026-05-26 09:30</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
           <t>Daniel Torres</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Dr. Diana Rodriguez</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>2026-05-26 09:30</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2870,22 +3900,32 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>1060793593</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Dr. Patricia Perez</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2026-05-20 10:00</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Sede Sur - Portal Norte</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
           <t>Tomas Garcia</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Dr. Patricia Perez</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>2026-05-20 10:00</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Sede Sur - Portal Norte</t>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2897,22 +3937,32 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>1087776473</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Dr. Hugo Flores</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2026-05-25 08:00</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
           <t>Patricia Rodriguez</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Dr. Hugo Flores</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>2026-05-25 08:00</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -2924,22 +3974,32 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>1066970088</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Dr. Ignacio Sanchez</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2026-05-27 18:00</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Clínica 100Digital</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
           <t>Eduardo Rivera</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Dr. Ignacio Sanchez</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>2026-05-27 18:00</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Clínica 100Digital</t>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2951,22 +4011,32 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
+          <t>1097965217</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Dr. Alejandro Morales</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2026-05-21 13:00</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Clínica 100Digital</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
           <t>Eduardo Morales</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Dr. Alejandro Morales</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>2026-05-21 13:00</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Clínica 100Digital</t>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
     </row>
@@ -2978,22 +4048,32 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>1042962502</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Dr. Patricia Rojas</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2026-05-23 12:30</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Sede Sur - Portal Norte</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
           <t>Sofia Ortiz</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Dr. Patricia Rojas</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>2026-05-23 12:30</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Sede Sur - Portal Norte</t>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -3005,22 +4085,32 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>1031734665</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Dr. Patricia Perez</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2026-05-25 15:00</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
           <t>Diana Ortiz</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Dr. Patricia Perez</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>2026-05-25 15:00</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -3032,22 +4122,32 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
+          <t>1087776473</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Dr. Beatriz Perez</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2026-05-20 14:30</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
           <t>Patricia Rodriguez</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Dr. Beatriz Perez</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>2026-05-20 14:30</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -3059,22 +4159,32 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>1034302379</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Dr. Gabriel Ramirez</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:00</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Sede Norte - Calle 127</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
           <t>Elena Ortiz</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Dr. Gabriel Ramirez</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>2026-05-22 13:00</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Sede Norte - Calle 127</t>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -3086,22 +4196,32 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>1056030198</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Dr. Gabriel Rojas</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2026-05-27 16:00</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Sede Sur - Portal Norte</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
           <t>Camila Ortiz</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Dr. Gabriel Rojas</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>2026-05-27 16:00</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Sede Sur - Portal Norte</t>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>
@@ -3113,22 +4233,32 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
+          <t>1018165720</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Dr. Diana Rodriguez</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2026-05-25 14:00</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Clínica 100Digital</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
           <t>Diana Cruz</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Dr. Diana Rodriguez</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>2026-05-25 14:00</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Clínica 100Digital</t>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
     </row>

</xml_diff>